<commit_message>
Updated the Zephyr testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -18,7 +18,419 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="137">
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:21:48</t>
+  </si>
+  <si>
+    <t>4661</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261009_102148_323.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:21:57</t>
+  </si>
+  <si>
+    <t>1740</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261009_102157_243.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:21:58</t>
+  </si>
+  <si>
+    <t>1436</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-4_20261009_102158_775.png</t>
+  </si>
+  <si>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:00</t>
+  </si>
+  <si>
+    <t>1610</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:03</t>
+  </si>
+  <si>
+    <t>1736</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:04</t>
+  </si>
+  <si>
+    <t>16677</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:05</t>
+  </si>
+  <si>
+    <t>985</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:08</t>
+  </si>
+  <si>
+    <t>1623</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:10</t>
+  </si>
+  <si>
+    <t>1047</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-2_20261009_102210_162.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:13</t>
+  </si>
+  <si>
+    <t>690</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-3_20261009_102213_102.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:26</t>
+  </si>
+  <si>
+    <t>16234</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 10:22:46</t>
+  </si>
+  <si>
+    <t>15839</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261009_102246_007.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:01:53</t>
+  </si>
+  <si>
+    <t>2672</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261009_190153_139.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:01:57</t>
+  </si>
+  <si>
+    <t>727</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261009_190157_003.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:03</t>
+  </si>
+  <si>
+    <t>1955</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-3_20261009_190203_040.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:06</t>
+  </si>
+  <si>
+    <t>736</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:08</t>
+  </si>
+  <si>
+    <t>1021</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-3_20261009_190208_359.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:09</t>
+  </si>
+  <si>
+    <t>15866</t>
+  </si>
+  <si>
+    <t>1414</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:13</t>
+  </si>
+  <si>
+    <t>1026</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-4_20261009_190213_394.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:28</t>
+  </si>
+  <si>
+    <t>16354</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:02:46</t>
+  </si>
+  <si>
+    <t>16250</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261009_190246_404.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:23:58</t>
+  </si>
+  <si>
+    <t>2938</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261009_192358_141.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:04</t>
+  </si>
+  <si>
+    <t>1324</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261009_192404_619.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:10</t>
+  </si>
+  <si>
+    <t>2338</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-3_20261009_192410_863.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:13</t>
+  </si>
+  <si>
+    <t>1254</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:15</t>
+  </si>
+  <si>
+    <t>1052</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-2_20261009_192415_317.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:16</t>
+  </si>
+  <si>
+    <t>17009</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:17</t>
+  </si>
+  <si>
+    <t>1056</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:20</t>
+  </si>
+  <si>
+    <t>762</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-4_20261009_192420_671.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:35</t>
+  </si>
+  <si>
+    <t>16041</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:24:56</t>
+  </si>
+  <si>
+    <t>16811</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261009_192456_349.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:22</t>
+  </si>
+  <si>
+    <t>3875</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261009_193222_507.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:28</t>
+  </si>
+  <si>
+    <t>1850</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261009_193228_385.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:35</t>
+  </si>
+  <si>
+    <t>1590</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-3_20261009_193235_567.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:36</t>
+  </si>
+  <si>
+    <t>1760</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:37</t>
+  </si>
+  <si>
+    <t>16366</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:40</t>
+  </si>
+  <si>
+    <t>1696</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-2_20261009_193240_026.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:42</t>
+  </si>
+  <si>
+    <t>716</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:46</t>
+  </si>
+  <si>
+    <t>702</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-4_20261009_193246_289.png</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:32:58</t>
+  </si>
+  <si>
+    <t>15970</t>
+  </si>
+  <si>
+    <t>09-Oct-2026 19:33:17</t>
+  </si>
+  <si>
+    <t>16167</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261009_193317_718.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:28</t>
+  </si>
+  <si>
+    <t>2944</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaArticleSearch_TestNG-test-WebRegressionSuite-3_20261012_122828_430.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:30</t>
+  </si>
+  <si>
+    <t>722</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHeroSection_TestNG-test-WebRegressionSuite-3_20261012_122830_223.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:32</t>
+  </si>
+  <si>
+    <t>982</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDocumentationPage_TestNG-test-WebRegressionSuite-3_20261012_122832_206.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:33</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:35</t>
+  </si>
+  <si>
+    <t>553</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:37</t>
+  </si>
+  <si>
+    <t>733</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaPortalTaglineInTitle_TestNG-test-WebRegressionSuite-3_20261012_122837_115.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:39</t>
+  </si>
+  <si>
+    <t>1113</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumDownloadsPageTitle_TestNG-test-WebRegressionSuite-3_20261012_122839_584.png</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:28:44</t>
+  </si>
+  <si>
+    <t>16103</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:29:00</t>
+  </si>
+  <si>
+    <t>15738</t>
+  </si>
+  <si>
+    <t>12-Oct-2026 12:29:17</t>
+  </si>
+  <si>
+    <t>15981</t>
+  </si>
+  <si>
+    <t>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaLanguageSelector_TestNG-test-WebRegressionSuite-1_20261012_122917_721.png</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -456,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.0"/>
@@ -547,13 +959,13 @@
         <v>PASS</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
-        <v>22-Sept-2026 20:40:52</v>
+        <v>12-Oct-2026 12:28:26</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
-        <v>7058</v>
+        <v>3792</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyAmazonHomePageTitle_TestNG-test-WebRegressionSuite-1_20260922_204051_740.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyAmazonHomePageTitle_TestNG-test-WebRegressionSuite-1_20261012_122826_748.png</v>
       </c>
     </row>
     <row r="3">
@@ -586,13 +998,13 @@
         <v>PASS</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
-        <v>22-Sept-2026 20:41:08</v>
+        <v>12-Oct-2026 12:28:44</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
-        <v>25340</v>
+        <v>21706</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyFlipkartHomePageTitle_TestNG-test-WebRegressionSuite-2_20260922_204108_511.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyFlipkartHomePageTitle_TestNG-test-WebRegressionSuite-2_20261012_122844_572.png</v>
       </c>
     </row>
     <row r="4">
@@ -625,13 +1037,13 @@
         <v>PASS</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <v>22-Sept-2026 20:40:47</v>
+        <v>12-Oct-2026 12:28:24</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
-        <v>4349</v>
+        <v>1574</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaHomePageTitle_TestNG-test-WebRegressionSuite-3_20260922_204047_093.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifyWikipediaHomePageTitle_TestNG-test-WebRegressionSuite-3_20261012_122824_006.png</v>
       </c>
     </row>
     <row r="5">
@@ -664,13 +1076,247 @@
         <v>PASS</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
-        <v>22-Sept-2026 20:41:01</v>
+        <v>12-Oct-2026 12:28:40</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
-        <v>18580</v>
+        <v>18100</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
-        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHomePageTitle_TestNG-test-WebRegressionSuite-4_20260922_204101_280.png</v>
+        <v>C:\Users\REDDY\Desktop\Git_Projects\Selenium-Java-Hybrid-Framework\test-output\Screenshots\verifySeleniumHomePageTitle_TestNG-test-WebRegressionSuite-4_20261012_122840_573.png</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC_005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Verify Wikipedia article search</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wikipedia.org</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Albert Einstein</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC_006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Verify Wikipedia language selector and featured languages</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wikipedia.org</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC_007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Verify Selenium home page hero section</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.selenium.dev</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC_008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Verify Selenium Documentation page</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.selenium.dev/documentation/</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC_009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Verify Wikipedia portal title tagline (expected FAIL)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wikipedia.org</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>The Free Encyclopedia</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC_010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Verify Selenium Downloads page title (expected FAIL)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.selenium.dev/downloads/</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Downloads Center</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>